<commit_message>
Update forest data - 2026-09-14 17:07
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4422" uniqueCount="2103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4432" uniqueCount="2106">
   <si>
     <t>link</t>
   </si>
@@ -6327,6 +6327,15 @@
   </si>
   <si>
     <t>3696-005-0125</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/ogre-and-reg/krapes-pag/annxl.html</t>
+  </si>
+  <si>
+    <t>74520080094</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/talsi-and-reg/virbu-pag/bhgkfj.html</t>
   </si>
 </sst>
 </file>
@@ -6739,7 +6748,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F882"/>
+  <dimension ref="A1:F883"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -24388,6 +24397,26 @@
       </c>
       <c r="F882" s="2">
         <v>46275.40347222222</v>
+      </c>
+    </row>
+    <row r="883" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A883" s="3" t="s">
+        <v>2100</v>
+      </c>
+      <c r="B883" s="4" t="s">
+        <v>533</v>
+      </c>
+      <c r="C883" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D883" s="4" t="s">
+        <v>2101</v>
+      </c>
+      <c r="E883" s="4" t="s">
+        <v>2102</v>
+      </c>
+      <c r="F883" s="2">
+        <v>46276.69861111111</v>
       </c>
     </row>
   </sheetData>
@@ -25273,6 +25302,7 @@
     <hyperlink ref="A880" r:id="rId879"/>
     <hyperlink ref="A881" r:id="rId880"/>
     <hyperlink ref="A882" r:id="rId881"/>
+    <hyperlink ref="A883" r:id="rId882"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -25284,7 +25314,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -25317,27 +25347,48 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>2100</v>
+        <v>2103</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>533</v>
+        <v>116</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>435</v>
+        <v>275</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>2101</v>
+        <v>1034</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>2102</v>
+        <v>2104</v>
       </c>
       <c r="F2" s="2">
-        <v>46276.69861111111</v>
+        <v>46277.65694444445</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>2105</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>1720</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>903</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>1721</v>
+      </c>
+      <c r="F3" s="2">
+        <v>46279.70763888889</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
+    <hyperlink ref="A3" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-09-15 15:47
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4432" uniqueCount="2106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4437" uniqueCount="2108">
   <si>
     <t>link</t>
   </si>
@@ -6336,6 +6336,12 @@
   </si>
   <si>
     <t>https://www.ss.com/msg/lv/real-estate/wood/talsi-and-reg/virbu-pag/bhgkfj.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/balvi-and-reg/viksnas-pag/ambmm.html</t>
+  </si>
+  <si>
+    <t>38940020163</t>
   </si>
 </sst>
 </file>
@@ -6748,7 +6754,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F883"/>
+  <dimension ref="A1:F885"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -24417,6 +24423,46 @@
       </c>
       <c r="F883" s="2">
         <v>46276.69861111111</v>
+      </c>
+    </row>
+    <row r="884" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A884" s="3" t="s">
+        <v>2103</v>
+      </c>
+      <c r="B884" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C884" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="D884" s="4" t="s">
+        <v>1034</v>
+      </c>
+      <c r="E884" s="4" t="s">
+        <v>2104</v>
+      </c>
+      <c r="F884" s="2">
+        <v>46277.65694444445</v>
+      </c>
+    </row>
+    <row r="885" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A885" s="3" t="s">
+        <v>2105</v>
+      </c>
+      <c r="B885" s="4" t="s">
+        <v>1720</v>
+      </c>
+      <c r="C885" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="D885" s="4" t="s">
+        <v>903</v>
+      </c>
+      <c r="E885" s="4" t="s">
+        <v>1721</v>
+      </c>
+      <c r="F885" s="2">
+        <v>46279.70763888889</v>
       </c>
     </row>
   </sheetData>
@@ -25303,6 +25349,8 @@
     <hyperlink ref="A881" r:id="rId880"/>
     <hyperlink ref="A882" r:id="rId881"/>
     <hyperlink ref="A883" r:id="rId882"/>
+    <hyperlink ref="A884" r:id="rId883"/>
+    <hyperlink ref="A885" r:id="rId884"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -25314,7 +25362,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -25347,48 +25395,27 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>2103</v>
+        <v>2106</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>116</v>
+        <v>91</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>275</v>
+        <v>28</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>1034</v>
+        <v>209</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>2104</v>
+        <v>2107</v>
       </c>
       <c r="F2" s="2">
-        <v>46277.65694444445</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>2105</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>1720</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>356</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>903</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>1721</v>
-      </c>
-      <c r="F3" s="2">
-        <v>46279.70763888889</v>
+        <v>46280.40416666667</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
-    <hyperlink ref="A3" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-09-16 15:39
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4437" uniqueCount="2108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4447" uniqueCount="2113">
   <si>
     <t>link</t>
   </si>
@@ -6342,6 +6342,21 @@
   </si>
   <si>
     <t>38940020163</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/cesis-and-reg/inesu-pag/ibbih.html</t>
+  </si>
+  <si>
+    <t>42540010107</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/preili-and-reg/galenu-pag/mgfic.html</t>
+  </si>
+  <si>
+    <t>2.67 ha.</t>
+  </si>
+  <si>
+    <t>7648-001-0141</t>
   </si>
 </sst>
 </file>
@@ -6754,7 +6769,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F885"/>
+  <dimension ref="A1:F886"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -24463,6 +24478,26 @@
       </c>
       <c r="F885" s="2">
         <v>46279.70763888889</v>
+      </c>
+    </row>
+    <row r="886" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A886" s="3" t="s">
+        <v>2106</v>
+      </c>
+      <c r="B886" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="C886" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D886" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="E886" s="4" t="s">
+        <v>2107</v>
+      </c>
+      <c r="F886" s="2">
+        <v>46280.40416666667</v>
       </c>
     </row>
   </sheetData>
@@ -25351,6 +25386,7 @@
     <hyperlink ref="A883" r:id="rId882"/>
     <hyperlink ref="A884" r:id="rId883"/>
     <hyperlink ref="A885" r:id="rId884"/>
+    <hyperlink ref="A886" r:id="rId885"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -25362,7 +25398,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -25395,27 +25431,48 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>2106</v>
+        <v>2108</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>91</v>
+        <v>43</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>28</v>
+        <v>63</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>209</v>
+        <v>186</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>2107</v>
+        <v>2109</v>
       </c>
       <c r="F2" s="2">
-        <v>46280.40416666667</v>
+        <v>46281.552777777775</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>2110</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>2111</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>2112</v>
+      </c>
+      <c r="F3" s="2">
+        <v>46281.43819444445</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
+    <hyperlink ref="A3" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-09-17 15:45
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -6769,7 +6769,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F886"/>
+  <dimension ref="A1:F888"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -24498,6 +24498,46 @@
       </c>
       <c r="F886" s="2">
         <v>46280.40416666667</v>
+      </c>
+    </row>
+    <row r="887" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A887" s="3" t="s">
+        <v>2108</v>
+      </c>
+      <c r="B887" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C887" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="D887" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="E887" s="4" t="s">
+        <v>2109</v>
+      </c>
+      <c r="F887" s="2">
+        <v>46281.552777777775</v>
+      </c>
+    </row>
+    <row r="888" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A888" s="3" t="s">
+        <v>2110</v>
+      </c>
+      <c r="B888" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C888" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="D888" s="4" t="s">
+        <v>2111</v>
+      </c>
+      <c r="E888" s="4" t="s">
+        <v>2112</v>
+      </c>
+      <c r="F888" s="2">
+        <v>46281.43819444445</v>
       </c>
     </row>
   </sheetData>
@@ -25387,6 +25427,8 @@
     <hyperlink ref="A884" r:id="rId883"/>
     <hyperlink ref="A885" r:id="rId884"/>
     <hyperlink ref="A886" r:id="rId885"/>
+    <hyperlink ref="A887" r:id="rId886"/>
+    <hyperlink ref="A888" r:id="rId887"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -25398,7 +25440,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -25429,51 +25471,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
-        <v>2108</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>2109</v>
-      </c>
-      <c r="F2" s="2">
-        <v>46281.552777777775</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>2110</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>284</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>2111</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>2112</v>
-      </c>
-      <c r="F3" s="2">
-        <v>46281.43819444445</v>
-      </c>
-    </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1"/>
-    <hyperlink ref="A3" r:id="rId2"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forest data - 2026-09-18 15:18
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4447" uniqueCount="2113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4457" uniqueCount="2118">
   <si>
     <t>link</t>
   </si>
@@ -6357,6 +6357,21 @@
   </si>
   <si>
     <t>7648-001-0141</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/daugavpils-and-reg/dubnas-pag/onoxi.html</t>
+  </si>
+  <si>
+    <t>44520040484</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/limbadzi-and-reg/liepupes-pag/imjgg.html</t>
+  </si>
+  <si>
+    <t>69 980 €</t>
+  </si>
+  <si>
+    <t>8.23 ha.</t>
   </si>
 </sst>
 </file>
@@ -25440,7 +25455,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -25471,7 +25486,51 @@
         <v>5</v>
       </c>
     </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>2113</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>1075</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>2114</v>
+      </c>
+      <c r="F2" s="2">
+        <v>46283.57986111111</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>2115</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>2116</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>2117</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>1535</v>
+      </c>
+      <c r="F3" s="2">
+        <v>46283.52569444444</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1"/>
+    <hyperlink ref="A3" r:id="rId2"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forest data - 2026-09-21 17:16
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -6784,7 +6784,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F888"/>
+  <dimension ref="A1:F890"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -24553,6 +24553,46 @@
       </c>
       <c r="F888" s="2">
         <v>46281.43819444445</v>
+      </c>
+    </row>
+    <row r="889" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A889" s="3" t="s">
+        <v>2113</v>
+      </c>
+      <c r="B889" s="4" t="s">
+        <v>1075</v>
+      </c>
+      <c r="C889" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="D889" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="E889" s="4" t="s">
+        <v>2114</v>
+      </c>
+      <c r="F889" s="2">
+        <v>46283.57986111111</v>
+      </c>
+    </row>
+    <row r="890" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A890" s="3" t="s">
+        <v>2115</v>
+      </c>
+      <c r="B890" s="4" t="s">
+        <v>2116</v>
+      </c>
+      <c r="C890" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="D890" s="4" t="s">
+        <v>2117</v>
+      </c>
+      <c r="E890" s="4" t="s">
+        <v>1535</v>
+      </c>
+      <c r="F890" s="2">
+        <v>46283.52569444444</v>
       </c>
     </row>
   </sheetData>
@@ -25444,6 +25484,8 @@
     <hyperlink ref="A886" r:id="rId885"/>
     <hyperlink ref="A887" r:id="rId886"/>
     <hyperlink ref="A888" r:id="rId887"/>
+    <hyperlink ref="A889" r:id="rId888"/>
+    <hyperlink ref="A890" r:id="rId889"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -25455,7 +25497,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -25486,51 +25528,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
-        <v>2113</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>1075</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>272</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>2114</v>
-      </c>
-      <c r="F2" s="2">
-        <v>46283.57986111111</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>2115</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>2116</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>208</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>2117</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>1535</v>
-      </c>
-      <c r="F3" s="2">
-        <v>46283.52569444444</v>
-      </c>
-    </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1"/>
-    <hyperlink ref="A3" r:id="rId2"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forest data - 2026-09-23 15:39
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4457" uniqueCount="2118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4467" uniqueCount="2123">
   <si>
     <t>link</t>
   </si>
@@ -6372,6 +6372,21 @@
   </si>
   <si>
     <t>8.23 ha.</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/rezekne-and-reg/makonkalna-pag/kxglo.html</t>
+  </si>
+  <si>
+    <t>78720100159</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/ventspils-and-reg/uzavas-pag/npjnb.html</t>
+  </si>
+  <si>
+    <t>1.53 ha.</t>
+  </si>
+  <si>
+    <t>98780070245</t>
   </si>
 </sst>
 </file>
@@ -25497,7 +25512,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -25528,7 +25543,51 @@
         <v>5</v>
       </c>
     </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>2118</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>2119</v>
+      </c>
+      <c r="F2" s="2">
+        <v>46288.054861111115</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>2120</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>969</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>404</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>2121</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>2122</v>
+      </c>
+      <c r="F3" s="2">
+        <v>46287.96319444444</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1"/>
+    <hyperlink ref="A3" r:id="rId2"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forest data - 2026-09-24 16:00
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4467" uniqueCount="2123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4477" uniqueCount="2128">
   <si>
     <t>link</t>
   </si>
@@ -6387,6 +6387,21 @@
   </si>
   <si>
     <t>98780070245</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/preili-and-reg/aglonas-pag/fmlbk.html</t>
+  </si>
+  <si>
+    <t>7.40 ha.</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/valmiera-and-reg/ramatas-pag/hdnco.html</t>
+  </si>
+  <si>
+    <t>37000 m²</t>
+  </si>
+  <si>
+    <t>96760080088</t>
   </si>
 </sst>
 </file>
@@ -6799,7 +6814,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F890"/>
+  <dimension ref="A1:F892"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -24608,6 +24623,46 @@
       </c>
       <c r="F890" s="2">
         <v>46283.52569444444</v>
+      </c>
+    </row>
+    <row r="891" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A891" s="3" t="s">
+        <v>2118</v>
+      </c>
+      <c r="B891" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C891" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="D891" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="E891" s="4" t="s">
+        <v>2119</v>
+      </c>
+      <c r="F891" s="2">
+        <v>46288.054861111115</v>
+      </c>
+    </row>
+    <row r="892" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A892" s="3" t="s">
+        <v>2120</v>
+      </c>
+      <c r="B892" s="4" t="s">
+        <v>969</v>
+      </c>
+      <c r="C892" s="4" t="s">
+        <v>404</v>
+      </c>
+      <c r="D892" s="4" t="s">
+        <v>2121</v>
+      </c>
+      <c r="E892" s="4" t="s">
+        <v>2122</v>
+      </c>
+      <c r="F892" s="2">
+        <v>46287.96319444444</v>
       </c>
     </row>
   </sheetData>
@@ -25501,6 +25556,8 @@
     <hyperlink ref="A888" r:id="rId887"/>
     <hyperlink ref="A889" r:id="rId888"/>
     <hyperlink ref="A890" r:id="rId889"/>
+    <hyperlink ref="A891" r:id="rId890"/>
+    <hyperlink ref="A892" r:id="rId891"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -25545,42 +25602,42 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>2118</v>
+        <v>2123</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>31</v>
+        <v>58</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>294</v>
+        <v>284</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>32</v>
+        <v>2124</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>2119</v>
+        <v>1893</v>
       </c>
       <c r="F2" s="2">
-        <v>46288.054861111115</v>
+        <v>46288.84861111111</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>2120</v>
+        <v>2125</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>969</v>
+        <v>43</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>404</v>
+        <v>396</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>2121</v>
+        <v>2126</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>2122</v>
+        <v>2127</v>
       </c>
       <c r="F3" s="2">
-        <v>46287.96319444444</v>
+        <v>46288.92708333333</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forest data - 2026-09-25 16:01
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4477" uniqueCount="2128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4482" uniqueCount="2129">
   <si>
     <t>link</t>
   </si>
@@ -6402,6 +6402,9 @@
   </si>
   <si>
     <t>96760080088</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/kuldiga-and-reg/ivandes-pag/kobcd.html</t>
   </si>
 </sst>
 </file>
@@ -6814,7 +6817,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F892"/>
+  <dimension ref="A1:F894"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -24663,6 +24666,46 @@
       </c>
       <c r="F892" s="2">
         <v>46287.96319444444</v>
+      </c>
+    </row>
+    <row r="893" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A893" s="3" t="s">
+        <v>2123</v>
+      </c>
+      <c r="B893" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="C893" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="D893" s="4" t="s">
+        <v>2124</v>
+      </c>
+      <c r="E893" s="4" t="s">
+        <v>1893</v>
+      </c>
+      <c r="F893" s="2">
+        <v>46288.84861111111</v>
+      </c>
+    </row>
+    <row r="894" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A894" s="3" t="s">
+        <v>2125</v>
+      </c>
+      <c r="B894" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C894" s="4" t="s">
+        <v>396</v>
+      </c>
+      <c r="D894" s="4" t="s">
+        <v>2126</v>
+      </c>
+      <c r="E894" s="4" t="s">
+        <v>2127</v>
+      </c>
+      <c r="F894" s="2">
+        <v>46288.92708333333</v>
       </c>
     </row>
   </sheetData>
@@ -25558,6 +25601,8 @@
     <hyperlink ref="A890" r:id="rId889"/>
     <hyperlink ref="A891" r:id="rId890"/>
     <hyperlink ref="A892" r:id="rId891"/>
+    <hyperlink ref="A893" r:id="rId892"/>
+    <hyperlink ref="A894" r:id="rId893"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -25569,7 +25614,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -25602,48 +25647,27 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>2123</v>
+        <v>2128</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>58</v>
+        <v>816</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>284</v>
+        <v>424</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>2124</v>
+        <v>17</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1893</v>
+        <v>1214</v>
       </c>
       <c r="F2" s="2">
-        <v>46288.84861111111</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>2125</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>396</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>2126</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>2127</v>
-      </c>
-      <c r="F3" s="2">
-        <v>46288.92708333333</v>
+        <v>46290.450694444444</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
-    <hyperlink ref="A3" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-09-28 18:50
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4482" uniqueCount="2129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4497" uniqueCount="2134">
   <si>
     <t>link</t>
   </si>
@@ -6405,6 +6405,21 @@
   </si>
   <si>
     <t>https://www.ss.com/msg/lv/real-estate/wood/kuldiga-and-reg/ivandes-pag/kobcd.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/jekabpils-and-reg/jekabpils/jkhji.html</t>
+  </si>
+  <si>
+    <t>56940090009</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/valmiera-and-reg/selu-pag/oblgo.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/ventspils-and-reg/varves-pag/nooxx.html</t>
+  </si>
+  <si>
+    <t>9884 001 0004</t>
   </si>
 </sst>
 </file>
@@ -6817,7 +6832,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F894"/>
+  <dimension ref="A1:F895"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -24706,6 +24721,26 @@
       </c>
       <c r="F894" s="2">
         <v>46288.92708333333</v>
+      </c>
+    </row>
+    <row r="895" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A895" s="3" t="s">
+        <v>2128</v>
+      </c>
+      <c r="B895" s="4" t="s">
+        <v>816</v>
+      </c>
+      <c r="C895" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="D895" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E895" s="4" t="s">
+        <v>1214</v>
+      </c>
+      <c r="F895" s="2">
+        <v>46290.450694444444</v>
       </c>
     </row>
   </sheetData>
@@ -25603,6 +25638,7 @@
     <hyperlink ref="A892" r:id="rId891"/>
     <hyperlink ref="A893" r:id="rId892"/>
     <hyperlink ref="A894" r:id="rId893"/>
+    <hyperlink ref="A895" r:id="rId894"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -25614,7 +25650,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -25647,27 +25683,69 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>2128</v>
+        <v>2129</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>816</v>
+        <v>58</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>424</v>
+        <v>127</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>17</v>
+        <v>59</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1214</v>
+        <v>2130</v>
       </c>
       <c r="F2" s="2">
-        <v>46290.450694444444</v>
+        <v>46292.589583333334</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>2131</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>271</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>396</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F3" s="2">
+        <v>46292.86875</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>2132</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>404</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>2133</v>
+      </c>
+      <c r="F4" s="2">
+        <v>46292.71944444445</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
+    <hyperlink ref="A3" r:id="rId2"/>
+    <hyperlink ref="A4" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-09-29 17:07
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4497" uniqueCount="2134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4502" uniqueCount="2136">
   <si>
     <t>link</t>
   </si>
@@ -6420,6 +6420,12 @@
   </si>
   <si>
     <t>9884 001 0004</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/valka-and-reg/blomes-pag/bxnehi.html</t>
+  </si>
+  <si>
+    <t>94460020024</t>
   </si>
 </sst>
 </file>
@@ -6832,7 +6838,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F895"/>
+  <dimension ref="A1:F898"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -24741,6 +24747,66 @@
       </c>
       <c r="F895" s="2">
         <v>46290.450694444444</v>
+      </c>
+    </row>
+    <row r="896" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A896" s="3" t="s">
+        <v>2129</v>
+      </c>
+      <c r="B896" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="C896" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="D896" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="E896" s="4" t="s">
+        <v>2130</v>
+      </c>
+      <c r="F896" s="2">
+        <v>46292.589583333334</v>
+      </c>
+    </row>
+    <row r="897" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A897" s="3" t="s">
+        <v>2131</v>
+      </c>
+      <c r="B897" s="4" t="s">
+        <v>271</v>
+      </c>
+      <c r="C897" s="4" t="s">
+        <v>396</v>
+      </c>
+      <c r="D897" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="E897" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F897" s="2">
+        <v>46292.86875</v>
+      </c>
+    </row>
+    <row r="898" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A898" s="3" t="s">
+        <v>2132</v>
+      </c>
+      <c r="B898" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="C898" s="4" t="s">
+        <v>404</v>
+      </c>
+      <c r="D898" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="E898" s="4" t="s">
+        <v>2133</v>
+      </c>
+      <c r="F898" s="2">
+        <v>46292.71944444445</v>
       </c>
     </row>
   </sheetData>
@@ -25639,6 +25705,9 @@
     <hyperlink ref="A893" r:id="rId892"/>
     <hyperlink ref="A894" r:id="rId893"/>
     <hyperlink ref="A895" r:id="rId894"/>
+    <hyperlink ref="A896" r:id="rId895"/>
+    <hyperlink ref="A897" r:id="rId896"/>
+    <hyperlink ref="A898" r:id="rId897"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -25650,7 +25719,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -25683,69 +25752,27 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>2129</v>
+        <v>2134</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>58</v>
+        <v>211</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>127</v>
+        <v>392</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>59</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>2130</v>
+        <v>2135</v>
       </c>
       <c r="F2" s="2">
-        <v>46292.589583333334</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>2131</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>271</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>396</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>272</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="F3" s="2">
-        <v>46292.86875</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>2132</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>467</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>404</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>272</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>2133</v>
-      </c>
-      <c r="F4" s="2">
-        <v>46292.71944444445</v>
+        <v>46294.45972222222</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
-    <hyperlink ref="A3" r:id="rId2"/>
-    <hyperlink ref="A4" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-09-30 17:05
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4502" uniqueCount="2136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4507" uniqueCount="2139">
   <si>
     <t>link</t>
   </si>
@@ -6426,6 +6426,15 @@
   </si>
   <si>
     <t>94460020024</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/madona-and-reg/liezeres-pag/icbck.html</t>
+  </si>
+  <si>
+    <t>47 900 €</t>
+  </si>
+  <si>
+    <t>7068 016 0094</t>
   </si>
 </sst>
 </file>
@@ -6838,7 +6847,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F898"/>
+  <dimension ref="A1:F899"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -24807,6 +24816,26 @@
       </c>
       <c r="F898" s="2">
         <v>46292.71944444445</v>
+      </c>
+    </row>
+    <row r="899" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A899" s="3" t="s">
+        <v>2134</v>
+      </c>
+      <c r="B899" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="C899" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="D899" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="E899" s="4" t="s">
+        <v>2135</v>
+      </c>
+      <c r="F899" s="2">
+        <v>46294.45972222222</v>
       </c>
     </row>
   </sheetData>
@@ -25708,6 +25737,7 @@
     <hyperlink ref="A896" r:id="rId895"/>
     <hyperlink ref="A897" r:id="rId896"/>
     <hyperlink ref="A898" r:id="rId897"/>
+    <hyperlink ref="A899" r:id="rId898"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -25752,22 +25782,22 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>2134</v>
+        <v>2136</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>211</v>
+        <v>2137</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>392</v>
+        <v>256</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>59</v>
+        <v>695</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>2135</v>
+        <v>2138</v>
       </c>
       <c r="F2" s="2">
-        <v>46294.45972222222</v>
+        <v>46295.73333333334</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forest data - 2026-10-01 17:37
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4507" uniqueCount="2139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4517" uniqueCount="2144">
   <si>
     <t>link</t>
   </si>
@@ -6435,6 +6435,21 @@
   </si>
   <si>
     <t>7068 016 0094</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/daugavpils-and-reg/malinovas-pag/kjpcl.html</t>
+  </si>
+  <si>
+    <t>44700040145</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/dobele-and-reg/dobeles-pag/ljnpd.html</t>
+  </si>
+  <si>
+    <t>199 000 €</t>
+  </si>
+  <si>
+    <t>46540030117.</t>
   </si>
 </sst>
 </file>
@@ -6847,7 +6862,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F899"/>
+  <dimension ref="A1:F900"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -24836,6 +24851,26 @@
       </c>
       <c r="F899" s="2">
         <v>46294.45972222222</v>
+      </c>
+    </row>
+    <row r="900" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A900" s="3" t="s">
+        <v>2136</v>
+      </c>
+      <c r="B900" s="4" t="s">
+        <v>2137</v>
+      </c>
+      <c r="C900" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="D900" s="4" t="s">
+        <v>695</v>
+      </c>
+      <c r="E900" s="4" t="s">
+        <v>2138</v>
+      </c>
+      <c r="F900" s="2">
+        <v>46295.73333333334</v>
       </c>
     </row>
   </sheetData>
@@ -25738,6 +25773,7 @@
     <hyperlink ref="A897" r:id="rId896"/>
     <hyperlink ref="A898" r:id="rId897"/>
     <hyperlink ref="A899" r:id="rId898"/>
+    <hyperlink ref="A900" r:id="rId899"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -25749,7 +25785,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -25782,27 +25818,48 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>2136</v>
+        <v>2139</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>2137</v>
+        <v>112</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>256</v>
+        <v>74</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>695</v>
+        <v>147</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>2138</v>
+        <v>2140</v>
       </c>
       <c r="F2" s="2">
-        <v>46295.73333333334</v>
+        <v>46296.50138888889</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>2141</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>2142</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>2143</v>
+      </c>
+      <c r="F3" s="2">
+        <v>46295.84861111111</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
+    <hyperlink ref="A3" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-10-02 16:54
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4517" uniqueCount="2144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4522" uniqueCount="2147">
   <si>
     <t>link</t>
   </si>
@@ -6450,6 +6450,15 @@
   </si>
   <si>
     <t>46540030117.</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/jekabpils-and-reg/saukas-pag/nooop.html</t>
+  </si>
+  <si>
+    <t>133 000 €</t>
+  </si>
+  <si>
+    <t>56880040075</t>
   </si>
 </sst>
 </file>
@@ -6862,7 +6871,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F900"/>
+  <dimension ref="A1:F902"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -24871,6 +24880,46 @@
       </c>
       <c r="F900" s="2">
         <v>46295.73333333334</v>
+      </c>
+    </row>
+    <row r="901" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A901" s="3" t="s">
+        <v>2139</v>
+      </c>
+      <c r="B901" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="C901" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="D901" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="E901" s="4" t="s">
+        <v>2140</v>
+      </c>
+      <c r="F901" s="2">
+        <v>46296.50138888889</v>
+      </c>
+    </row>
+    <row r="902" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A902" s="3" t="s">
+        <v>2141</v>
+      </c>
+      <c r="B902" s="4" t="s">
+        <v>2142</v>
+      </c>
+      <c r="C902" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="D902" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E902" s="4" t="s">
+        <v>2143</v>
+      </c>
+      <c r="F902" s="2">
+        <v>46295.84861111111</v>
       </c>
     </row>
   </sheetData>
@@ -25774,6 +25823,8 @@
     <hyperlink ref="A898" r:id="rId897"/>
     <hyperlink ref="A899" r:id="rId898"/>
     <hyperlink ref="A900" r:id="rId899"/>
+    <hyperlink ref="A901" r:id="rId900"/>
+    <hyperlink ref="A902" r:id="rId901"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -25785,7 +25836,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -25818,48 +25869,27 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>2139</v>
+        <v>2144</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>112</v>
+        <v>2145</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>74</v>
+        <v>127</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>147</v>
+        <v>699</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>2140</v>
+        <v>2146</v>
       </c>
       <c r="F2" s="2">
-        <v>46296.50138888889</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>2141</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>2142</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>117</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>2143</v>
-      </c>
-      <c r="F3" s="2">
-        <v>46295.84861111111</v>
+        <v>46297.60902777778</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
-    <hyperlink ref="A3" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-10-05 19:50
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4522" uniqueCount="2147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4527" uniqueCount="2149">
   <si>
     <t>link</t>
   </si>
@@ -6459,6 +6459,12 @@
   </si>
   <si>
     <t>56880040075</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/limbadzi-and-reg/limbazu-pag/dgbik.html</t>
+  </si>
+  <si>
+    <t>6640070005</t>
   </si>
 </sst>
 </file>
@@ -6871,7 +6877,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F902"/>
+  <dimension ref="A1:F903"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -24920,6 +24926,26 @@
       </c>
       <c r="F902" s="2">
         <v>46295.84861111111</v>
+      </c>
+    </row>
+    <row r="903" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A903" s="3" t="s">
+        <v>2144</v>
+      </c>
+      <c r="B903" s="4" t="s">
+        <v>2145</v>
+      </c>
+      <c r="C903" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="D903" s="4" t="s">
+        <v>699</v>
+      </c>
+      <c r="E903" s="4" t="s">
+        <v>2146</v>
+      </c>
+      <c r="F903" s="2">
+        <v>46297.60902777778</v>
       </c>
     </row>
   </sheetData>
@@ -25825,6 +25851,7 @@
     <hyperlink ref="A900" r:id="rId899"/>
     <hyperlink ref="A901" r:id="rId900"/>
     <hyperlink ref="A902" r:id="rId901"/>
+    <hyperlink ref="A903" r:id="rId902"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -25869,22 +25896,22 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>2144</v>
+        <v>2147</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>2145</v>
+        <v>477</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>127</v>
+        <v>208</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>699</v>
+        <v>1558</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>2146</v>
+        <v>2148</v>
       </c>
       <c r="F2" s="2">
-        <v>46297.60902777778</v>
+        <v>46300.45625</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forest data - 2026-10-06 17:29
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4527" uniqueCount="2149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4537" uniqueCount="2153">
   <si>
     <t>link</t>
   </si>
@@ -6465,6 +6465,18 @@
   </si>
   <si>
     <t>6640070005</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/gulbene-and-reg/daukstu-pag/oldce.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/limbadzi-and-reg/staicele/gdghb.html</t>
+  </si>
+  <si>
+    <t>250 000 €</t>
+  </si>
+  <si>
+    <t>66370020120</t>
   </si>
 </sst>
 </file>
@@ -6877,7 +6889,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F903"/>
+  <dimension ref="A1:F904"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -24946,6 +24958,26 @@
       </c>
       <c r="F903" s="2">
         <v>46297.60902777778</v>
+      </c>
+    </row>
+    <row r="904" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A904" s="3" t="s">
+        <v>2147</v>
+      </c>
+      <c r="B904" s="4" t="s">
+        <v>477</v>
+      </c>
+      <c r="C904" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="D904" s="4" t="s">
+        <v>1558</v>
+      </c>
+      <c r="E904" s="4" t="s">
+        <v>2148</v>
+      </c>
+      <c r="F904" s="2">
+        <v>46300.45625</v>
       </c>
     </row>
   </sheetData>
@@ -25852,6 +25884,7 @@
     <hyperlink ref="A901" r:id="rId900"/>
     <hyperlink ref="A902" r:id="rId901"/>
     <hyperlink ref="A903" r:id="rId902"/>
+    <hyperlink ref="A904" r:id="rId903"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -25863,7 +25896,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -25896,27 +25929,48 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>2147</v>
+        <v>2149</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>477</v>
+        <v>106</v>
       </c>
       <c r="C2" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>1604</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>1605</v>
+      </c>
+      <c r="F2" s="2">
+        <v>46301.82638888889</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>2150</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>2151</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>208</v>
       </c>
-      <c r="D2" s="4" t="s">
-        <v>1558</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>2148</v>
-      </c>
-      <c r="F2" s="2">
-        <v>46300.45625</v>
+      <c r="D3" s="4" t="s">
+        <v>2071</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>2152</v>
+      </c>
+      <c r="F3" s="2">
+        <v>46301.83125</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
+    <hyperlink ref="A3" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-10-07 18:01
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4537" uniqueCount="2153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4547" uniqueCount="2157">
   <si>
     <t>link</t>
   </si>
@@ -6477,6 +6477,18 @@
   </si>
   <si>
     <t>66370020120</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/daugavpils-and-reg/demenes-pag/obgdj.html</t>
+  </si>
+  <si>
+    <t>8 800 €</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/kraslava-and-reg/andzelu-pag/dmlek.html</t>
+  </si>
+  <si>
+    <t>60440030037</t>
   </si>
 </sst>
 </file>
@@ -6889,7 +6901,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F904"/>
+  <dimension ref="A1:F906"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -24978,6 +24990,46 @@
       </c>
       <c r="F904" s="2">
         <v>46300.45625</v>
+      </c>
+    </row>
+    <row r="905" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A905" s="3" t="s">
+        <v>2149</v>
+      </c>
+      <c r="B905" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C905" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="D905" s="4" t="s">
+        <v>1604</v>
+      </c>
+      <c r="E905" s="4" t="s">
+        <v>1605</v>
+      </c>
+      <c r="F905" s="2">
+        <v>46301.82638888889</v>
+      </c>
+    </row>
+    <row r="906" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A906" s="3" t="s">
+        <v>2150</v>
+      </c>
+      <c r="B906" s="4" t="s">
+        <v>2151</v>
+      </c>
+      <c r="C906" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="D906" s="4" t="s">
+        <v>2071</v>
+      </c>
+      <c r="E906" s="4" t="s">
+        <v>2152</v>
+      </c>
+      <c r="F906" s="2">
+        <v>46301.83125</v>
       </c>
     </row>
   </sheetData>
@@ -25885,6 +25937,8 @@
     <hyperlink ref="A902" r:id="rId901"/>
     <hyperlink ref="A903" r:id="rId902"/>
     <hyperlink ref="A904" r:id="rId903"/>
+    <hyperlink ref="A905" r:id="rId904"/>
+    <hyperlink ref="A906" r:id="rId905"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -25929,42 +25983,42 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>2149</v>
+        <v>2153</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>106</v>
+        <v>2154</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>124</v>
+        <v>74</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>1604</v>
+        <v>36</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>1605</v>
+        <v>25</v>
       </c>
       <c r="F2" s="2">
-        <v>46301.82638888889</v>
+        <v>46302.629166666666</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>2150</v>
+        <v>2155</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>2151</v>
+        <v>88</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>208</v>
+        <v>146</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>2071</v>
+        <v>1259</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>2152</v>
+        <v>2156</v>
       </c>
       <c r="F3" s="2">
-        <v>46301.83125</v>
+        <v>46302.40347222222</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forest data - 2026-10-08 18:04
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4547" uniqueCount="2157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4557" uniqueCount="2161">
   <si>
     <t>link</t>
   </si>
@@ -6489,6 +6489,18 @@
   </si>
   <si>
     <t>60440030037</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/preili-and-reg/riebinu-pag/fjenh.html</t>
+  </si>
+  <si>
+    <t>76620040092</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/valka-and-reg/blomes-pag/bxodbj.html</t>
+  </si>
+  <si>
+    <t>94460020040</t>
   </si>
 </sst>
 </file>
@@ -6901,7 +6913,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F906"/>
+  <dimension ref="A1:F908"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -25030,6 +25042,46 @@
       </c>
       <c r="F906" s="2">
         <v>46301.83125</v>
+      </c>
+    </row>
+    <row r="907" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A907" s="3" t="s">
+        <v>2153</v>
+      </c>
+      <c r="B907" s="4" t="s">
+        <v>2154</v>
+      </c>
+      <c r="C907" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="D907" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E907" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F907" s="2">
+        <v>46302.629166666666</v>
+      </c>
+    </row>
+    <row r="908" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A908" s="3" t="s">
+        <v>2155</v>
+      </c>
+      <c r="B908" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="C908" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="D908" s="4" t="s">
+        <v>1259</v>
+      </c>
+      <c r="E908" s="4" t="s">
+        <v>2156</v>
+      </c>
+      <c r="F908" s="2">
+        <v>46302.40347222222</v>
       </c>
     </row>
   </sheetData>
@@ -25939,6 +25991,8 @@
     <hyperlink ref="A904" r:id="rId903"/>
     <hyperlink ref="A905" r:id="rId904"/>
     <hyperlink ref="A906" r:id="rId905"/>
+    <hyperlink ref="A907" r:id="rId906"/>
+    <hyperlink ref="A908" r:id="rId907"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -25983,42 +26037,42 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>2153</v>
+        <v>2157</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>2154</v>
+        <v>185</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>74</v>
+        <v>284</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>36</v>
+        <v>186</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>25</v>
+        <v>2158</v>
       </c>
       <c r="F2" s="2">
-        <v>46302.629166666666</v>
+        <v>46303.48472222222</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>2155</v>
+        <v>2159</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>88</v>
+        <v>650</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>146</v>
+        <v>392</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>1259</v>
+        <v>959</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>2156</v>
+        <v>2160</v>
       </c>
       <c r="F3" s="2">
-        <v>46302.40347222222</v>
+        <v>46302.96805555555</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forest data - 2026-10-09 17:38
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4557" uniqueCount="2161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4567" uniqueCount="2164">
   <si>
     <t>link</t>
   </si>
@@ -6501,6 +6501,15 @@
   </si>
   <si>
     <t>94460020040</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aluksne-and-reg/aluksne/pkhbx.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/liepaja-and-reg/aizputes-pag/beoixm.html</t>
+  </si>
+  <si>
+    <t>64420050259</t>
   </si>
 </sst>
 </file>
@@ -6913,7 +6922,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F908"/>
+  <dimension ref="A1:F910"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -25082,6 +25091,46 @@
       </c>
       <c r="F908" s="2">
         <v>46302.40347222222</v>
+      </c>
+    </row>
+    <row r="909" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A909" s="3" t="s">
+        <v>2157</v>
+      </c>
+      <c r="B909" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="C909" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="D909" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="E909" s="4" t="s">
+        <v>2158</v>
+      </c>
+      <c r="F909" s="2">
+        <v>46303.48472222222</v>
+      </c>
+    </row>
+    <row r="910" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A910" s="3" t="s">
+        <v>2159</v>
+      </c>
+      <c r="B910" s="4" t="s">
+        <v>650</v>
+      </c>
+      <c r="C910" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="D910" s="4" t="s">
+        <v>959</v>
+      </c>
+      <c r="E910" s="4" t="s">
+        <v>2160</v>
+      </c>
+      <c r="F910" s="2">
+        <v>46302.96805555555</v>
       </c>
     </row>
   </sheetData>
@@ -25993,6 +26042,8 @@
     <hyperlink ref="A906" r:id="rId905"/>
     <hyperlink ref="A907" r:id="rId906"/>
     <hyperlink ref="A908" r:id="rId907"/>
+    <hyperlink ref="A909" r:id="rId908"/>
+    <hyperlink ref="A910" r:id="rId909"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -26037,42 +26088,42 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>2157</v>
+        <v>2161</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>185</v>
+        <v>25</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>284</v>
+        <v>435</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>186</v>
+        <v>162</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>2158</v>
+        <v>25</v>
       </c>
       <c r="F2" s="2">
-        <v>46303.48472222222</v>
+        <v>46303.88402777778</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>2159</v>
+        <v>2162</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>650</v>
+        <v>1935</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>392</v>
+        <v>190</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>959</v>
+        <v>272</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>2160</v>
+        <v>2163</v>
       </c>
       <c r="F3" s="2">
-        <v>46302.96805555555</v>
+        <v>46303.88888888889</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update forest data - 2026-10-12 20:32
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4567" uniqueCount="2164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4597" uniqueCount="2174">
   <si>
     <t>link</t>
   </si>
@@ -6510,6 +6510,36 @@
   </si>
   <si>
     <t>64420050259</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aizkraukle-and-reg/jaunjelgavas-l-t/jppeg.html</t>
+  </si>
+  <si>
+    <t>32070010099</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aluksne-and-reg/ilzenes-pag/oihgc.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aluksne-and-reg/jaunlaicenes-pag/bdxkbd.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/cesis-and-reg/drabesu-pag/kgfdh.html</t>
+  </si>
+  <si>
+    <t>188 888 €</t>
+  </si>
+  <si>
+    <t>42460080051</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/madona-and-reg/praulienas-pag/mhhnl.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/talsi-and-reg/valdgales-pag/hjiih.html</t>
+  </si>
+  <si>
+    <t>88920120069</t>
   </si>
 </sst>
 </file>
@@ -6922,7 +6952,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F910"/>
+  <dimension ref="A1:F912"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -25131,6 +25161,46 @@
       </c>
       <c r="F910" s="2">
         <v>46302.96805555555</v>
+      </c>
+    </row>
+    <row r="911" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A911" s="3" t="s">
+        <v>2161</v>
+      </c>
+      <c r="B911" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C911" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D911" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="E911" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F911" s="2">
+        <v>46303.88402777778</v>
+      </c>
+    </row>
+    <row r="912" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A912" s="3" t="s">
+        <v>2162</v>
+      </c>
+      <c r="B912" s="4" t="s">
+        <v>1935</v>
+      </c>
+      <c r="C912" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="D912" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="E912" s="4" t="s">
+        <v>2163</v>
+      </c>
+      <c r="F912" s="2">
+        <v>46303.88888888889</v>
       </c>
     </row>
   </sheetData>
@@ -26044,6 +26114,8 @@
     <hyperlink ref="A908" r:id="rId907"/>
     <hyperlink ref="A909" r:id="rId908"/>
     <hyperlink ref="A910" r:id="rId909"/>
+    <hyperlink ref="A911" r:id="rId910"/>
+    <hyperlink ref="A912" r:id="rId911"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -26055,7 +26127,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -26088,48 +26160,132 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>2161</v>
+        <v>2164</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>25</v>
+        <v>650</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>435</v>
+        <v>8</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>162</v>
+        <v>59</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>25</v>
+        <v>2165</v>
       </c>
       <c r="F2" s="2">
-        <v>46303.88402777778</v>
+        <v>46305.57916666666</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>2162</v>
+        <v>2166</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>1935</v>
+        <v>25</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>190</v>
+        <v>435</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>272</v>
+        <v>25</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>2163</v>
+        <v>25</v>
       </c>
       <c r="F3" s="2">
-        <v>46303.88888888889</v>
+        <v>46307.38125</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>2167</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F4" s="2">
+        <v>46304.888194444444</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>2168</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>2169</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>2170</v>
+      </c>
+      <c r="F5" s="2">
+        <v>46305.63125</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>2171</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>654</v>
+      </c>
+      <c r="F6" s="2">
+        <v>46307.663888888885</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>2172</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>2173</v>
+      </c>
+      <c r="F7" s="2">
+        <v>46307.59166666667</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
     <hyperlink ref="A3" r:id="rId2"/>
+    <hyperlink ref="A4" r:id="rId3"/>
+    <hyperlink ref="A5" r:id="rId4"/>
+    <hyperlink ref="A6" r:id="rId5"/>
+    <hyperlink ref="A7" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-10-13 18:36
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4597" uniqueCount="2174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4607" uniqueCount="2177">
   <si>
     <t>link</t>
   </si>
@@ -6540,6 +6540,15 @@
   </si>
   <si>
     <t>88920120069</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aluksne-and-reg/pededzes-pag/bxhejn.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/madona-and-reg/vestienas-pag/kegjf.html</t>
+  </si>
+  <si>
+    <t>70960070353</t>
   </si>
 </sst>
 </file>
@@ -6952,7 +6961,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F912"/>
+  <dimension ref="A1:F918"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -25201,6 +25210,126 @@
       </c>
       <c r="F912" s="2">
         <v>46303.88888888889</v>
+      </c>
+    </row>
+    <row r="913" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A913" s="3" t="s">
+        <v>2164</v>
+      </c>
+      <c r="B913" s="4" t="s">
+        <v>650</v>
+      </c>
+      <c r="C913" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D913" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="E913" s="4" t="s">
+        <v>2165</v>
+      </c>
+      <c r="F913" s="2">
+        <v>46305.57916666666</v>
+      </c>
+    </row>
+    <row r="914" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A914" s="3" t="s">
+        <v>2166</v>
+      </c>
+      <c r="B914" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C914" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D914" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E914" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F914" s="2">
+        <v>46307.38125</v>
+      </c>
+    </row>
+    <row r="915" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A915" s="3" t="s">
+        <v>2167</v>
+      </c>
+      <c r="B915" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C915" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D915" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E915" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F915" s="2">
+        <v>46304.888194444444</v>
+      </c>
+    </row>
+    <row r="916" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A916" s="3" t="s">
+        <v>2168</v>
+      </c>
+      <c r="B916" s="4" t="s">
+        <v>2169</v>
+      </c>
+      <c r="C916" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="D916" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E916" s="4" t="s">
+        <v>2170</v>
+      </c>
+      <c r="F916" s="2">
+        <v>46305.63125</v>
+      </c>
+    </row>
+    <row r="917" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A917" s="3" t="s">
+        <v>2171</v>
+      </c>
+      <c r="B917" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="C917" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="D917" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="E917" s="4" t="s">
+        <v>654</v>
+      </c>
+      <c r="F917" s="2">
+        <v>46307.663888888885</v>
+      </c>
+    </row>
+    <row r="918" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A918" s="3" t="s">
+        <v>2172</v>
+      </c>
+      <c r="B918" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C918" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="D918" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="E918" s="4" t="s">
+        <v>2173</v>
+      </c>
+      <c r="F918" s="2">
+        <v>46307.59166666667</v>
       </c>
     </row>
   </sheetData>
@@ -26116,6 +26245,12 @@
     <hyperlink ref="A910" r:id="rId909"/>
     <hyperlink ref="A911" r:id="rId910"/>
     <hyperlink ref="A912" r:id="rId911"/>
+    <hyperlink ref="A913" r:id="rId912"/>
+    <hyperlink ref="A914" r:id="rId913"/>
+    <hyperlink ref="A915" r:id="rId914"/>
+    <hyperlink ref="A916" r:id="rId915"/>
+    <hyperlink ref="A917" r:id="rId916"/>
+    <hyperlink ref="A918" r:id="rId917"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -26127,7 +26262,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -26160,132 +26295,48 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>2164</v>
+        <v>2174</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>650</v>
+        <v>25</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>8</v>
+        <v>435</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>59</v>
+        <v>25</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>2165</v>
+        <v>25</v>
       </c>
       <c r="F2" s="2">
-        <v>46305.57916666666</v>
+        <v>46308.47152777778</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>2166</v>
+        <v>2175</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>25</v>
+        <v>337</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>435</v>
+        <v>256</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>25</v>
+        <v>553</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>25</v>
+        <v>2176</v>
       </c>
       <c r="F3" s="2">
-        <v>46307.38125</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>2167</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>435</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="F4" s="2">
-        <v>46304.888194444444</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>2168</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>2169</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>2170</v>
-      </c>
-      <c r="F5" s="2">
-        <v>46305.63125</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>2171</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>256</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>154</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>654</v>
-      </c>
-      <c r="F6" s="2">
-        <v>46307.663888888885</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
-        <v>2172</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>356</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>2173</v>
-      </c>
-      <c r="F7" s="2">
-        <v>46307.59166666667</v>
+        <v>46308.459027777775</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
     <hyperlink ref="A3" r:id="rId2"/>
-    <hyperlink ref="A4" r:id="rId3"/>
-    <hyperlink ref="A5" r:id="rId4"/>
-    <hyperlink ref="A6" r:id="rId5"/>
-    <hyperlink ref="A7" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-10-14 16:04
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4607" uniqueCount="2177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4622" uniqueCount="2182">
   <si>
     <t>link</t>
   </si>
@@ -6549,6 +6549,21 @@
   </si>
   <si>
     <t>70960070353</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aizkraukle-and-reg/sunakstes-pag/bbcfm.html</t>
+  </si>
+  <si>
+    <t>54 ha.</t>
+  </si>
+  <si>
+    <t>32860020249</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aluksne-and-reg/aluksne/pcdlp.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aluksne-and-reg/veclaicenes-pag/bljxfm.html</t>
   </si>
 </sst>
 </file>
@@ -6961,7 +6976,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F918"/>
+  <dimension ref="A1:F920"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -25330,6 +25345,46 @@
       </c>
       <c r="F918" s="2">
         <v>46307.59166666667</v>
+      </c>
+    </row>
+    <row r="919" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A919" s="3" t="s">
+        <v>2174</v>
+      </c>
+      <c r="B919" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C919" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D919" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E919" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F919" s="2">
+        <v>46308.47152777778</v>
+      </c>
+    </row>
+    <row r="920" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A920" s="3" t="s">
+        <v>2175</v>
+      </c>
+      <c r="B920" s="4" t="s">
+        <v>337</v>
+      </c>
+      <c r="C920" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="D920" s="4" t="s">
+        <v>553</v>
+      </c>
+      <c r="E920" s="4" t="s">
+        <v>2176</v>
+      </c>
+      <c r="F920" s="2">
+        <v>46308.459027777775</v>
       </c>
     </row>
   </sheetData>
@@ -26251,6 +26306,8 @@
     <hyperlink ref="A916" r:id="rId915"/>
     <hyperlink ref="A917" r:id="rId916"/>
     <hyperlink ref="A918" r:id="rId917"/>
+    <hyperlink ref="A919" r:id="rId918"/>
+    <hyperlink ref="A920" r:id="rId919"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -26262,7 +26319,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -26295,48 +26352,69 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>2174</v>
+        <v>2177</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>25</v>
+        <v>513</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>435</v>
+        <v>8</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>25</v>
+        <v>2178</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>25</v>
+        <v>2179</v>
       </c>
       <c r="F2" s="2">
-        <v>46308.47152777778</v>
+        <v>46309.55694444444</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>2175</v>
+        <v>2180</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>337</v>
+        <v>25</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>256</v>
+        <v>435</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>553</v>
+        <v>25</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>2176</v>
+        <v>25</v>
       </c>
       <c r="F3" s="2">
-        <v>46308.459027777775</v>
+        <v>46309.78333333333</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>2181</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F4" s="2">
+        <v>46309.396527777775</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
     <hyperlink ref="A3" r:id="rId2"/>
+    <hyperlink ref="A4" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-10-15 15:53
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4622" uniqueCount="2182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4627" uniqueCount="2184">
   <si>
     <t>link</t>
   </si>
@@ -6564,6 +6564,12 @@
   </si>
   <si>
     <t>https://www.ss.com/msg/lv/real-estate/wood/aluksne-and-reg/veclaicenes-pag/bljxfm.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/kuldiga-and-reg/edoles-pag/jhnce.html</t>
+  </si>
+  <si>
+    <t>62460060134</t>
   </si>
 </sst>
 </file>
@@ -6976,7 +6982,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F920"/>
+  <dimension ref="A1:F923"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -25385,6 +25391,66 @@
       </c>
       <c r="F920" s="2">
         <v>46308.459027777775</v>
+      </c>
+    </row>
+    <row r="921" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A921" s="3" t="s">
+        <v>2177</v>
+      </c>
+      <c r="B921" s="4" t="s">
+        <v>513</v>
+      </c>
+      <c r="C921" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D921" s="4" t="s">
+        <v>2178</v>
+      </c>
+      <c r="E921" s="4" t="s">
+        <v>2179</v>
+      </c>
+      <c r="F921" s="2">
+        <v>46309.55694444444</v>
+      </c>
+    </row>
+    <row r="922" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A922" s="3" t="s">
+        <v>2180</v>
+      </c>
+      <c r="B922" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C922" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D922" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E922" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F922" s="2">
+        <v>46309.78333333333</v>
+      </c>
+    </row>
+    <row r="923" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A923" s="3" t="s">
+        <v>2181</v>
+      </c>
+      <c r="B923" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C923" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D923" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E923" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F923" s="2">
+        <v>46309.396527777775</v>
       </c>
     </row>
   </sheetData>
@@ -26308,6 +26374,9 @@
     <hyperlink ref="A918" r:id="rId917"/>
     <hyperlink ref="A919" r:id="rId918"/>
     <hyperlink ref="A920" r:id="rId919"/>
+    <hyperlink ref="A921" r:id="rId920"/>
+    <hyperlink ref="A922" r:id="rId921"/>
+    <hyperlink ref="A923" r:id="rId922"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -26319,7 +26388,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -26352,69 +26421,27 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>2177</v>
+        <v>2182</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>513</v>
+        <v>204</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>8</v>
+        <v>424</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>2178</v>
+        <v>53</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>2179</v>
+        <v>2183</v>
       </c>
       <c r="F2" s="2">
-        <v>46309.55694444444</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>2180</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>435</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="F3" s="2">
-        <v>46309.78333333333</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>2181</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>435</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="F4" s="2">
-        <v>46309.396527777775</v>
+        <v>46309.82291666667</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
-    <hyperlink ref="A3" r:id="rId2"/>
-    <hyperlink ref="A4" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-10-16 15:40
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4627" uniqueCount="2184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4642" uniqueCount="2189">
   <si>
     <t>link</t>
   </si>
@@ -6570,6 +6570,21 @@
   </si>
   <si>
     <t>62460060134</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aluksne-and-reg/veclaicenes-pag/bdildf.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/bauska-and-reg/brunavas-pag/npeed.html</t>
+  </si>
+  <si>
+    <t>40460090068</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/liepaja-and-reg/gaviezes-pag/joeie.html</t>
+  </si>
+  <si>
+    <t>64560060036</t>
   </si>
 </sst>
 </file>
@@ -6982,7 +6997,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F923"/>
+  <dimension ref="A1:F924"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -25451,6 +25466,26 @@
       </c>
       <c r="F923" s="2">
         <v>46309.396527777775</v>
+      </c>
+    </row>
+    <row r="924" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A924" s="3" t="s">
+        <v>2182</v>
+      </c>
+      <c r="B924" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="C924" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="D924" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="E924" s="4" t="s">
+        <v>2183</v>
+      </c>
+      <c r="F924" s="2">
+        <v>46309.82291666667</v>
       </c>
     </row>
   </sheetData>
@@ -26377,6 +26412,7 @@
     <hyperlink ref="A921" r:id="rId920"/>
     <hyperlink ref="A922" r:id="rId921"/>
     <hyperlink ref="A923" r:id="rId922"/>
+    <hyperlink ref="A924" r:id="rId923"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -26388,7 +26424,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -26421,27 +26457,69 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>2182</v>
+        <v>2184</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>204</v>
+        <v>25</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>424</v>
+        <v>435</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>53</v>
+        <v>25</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>2183</v>
+        <v>25</v>
       </c>
       <c r="F2" s="2">
-        <v>46309.82291666667</v>
+        <v>46311.226388888885</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>2185</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>290</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>2186</v>
+      </c>
+      <c r="F3" s="2">
+        <v>46311.694444444445</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>2187</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>1610</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>2188</v>
+      </c>
+      <c r="F4" s="2">
+        <v>46311.51041666667</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1"/>
+    <hyperlink ref="A3" r:id="rId2"/>
+    <hyperlink ref="A4" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-10-19 17:54
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4642" uniqueCount="2189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4672" uniqueCount="2199">
   <si>
     <t>link</t>
   </si>
@@ -6585,6 +6585,36 @@
   </si>
   <si>
     <t>64560060036</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aizkraukle-and-reg/pilskalnes-pag/chgel.html</t>
+  </si>
+  <si>
+    <t>2.37 ha.</t>
+  </si>
+  <si>
+    <t>32740050052</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aluksne-and-reg/trapenes-pag/mkelj.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aluksne-and-reg/aluksne/epgog.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aluksne-and-reg/pededzes-pag/bxcxkk.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/madona-and-reg/liezeres-pag/fepfg.html</t>
+  </si>
+  <si>
+    <t>70680160066</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/rezekne-and-reg/kantinieku-pag/aopmp.html</t>
+  </si>
+  <si>
+    <t>78600020057</t>
   </si>
 </sst>
 </file>
@@ -6997,7 +7027,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F924"/>
+  <dimension ref="A1:F927"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -25486,6 +25516,66 @@
       </c>
       <c r="F924" s="2">
         <v>46309.82291666667</v>
+      </c>
+    </row>
+    <row r="925" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A925" s="3" t="s">
+        <v>2184</v>
+      </c>
+      <c r="B925" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C925" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D925" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E925" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F925" s="2">
+        <v>46311.226388888885</v>
+      </c>
+    </row>
+    <row r="926" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A926" s="3" t="s">
+        <v>2185</v>
+      </c>
+      <c r="B926" s="4" t="s">
+        <v>290</v>
+      </c>
+      <c r="C926" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="D926" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="E926" s="4" t="s">
+        <v>2186</v>
+      </c>
+      <c r="F926" s="2">
+        <v>46311.694444444445</v>
+      </c>
+    </row>
+    <row r="927" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A927" s="3" t="s">
+        <v>2187</v>
+      </c>
+      <c r="B927" s="4" t="s">
+        <v>1610</v>
+      </c>
+      <c r="C927" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="D927" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="E927" s="4" t="s">
+        <v>2188</v>
+      </c>
+      <c r="F927" s="2">
+        <v>46311.51041666667</v>
       </c>
     </row>
   </sheetData>
@@ -26413,6 +26503,9 @@
     <hyperlink ref="A922" r:id="rId921"/>
     <hyperlink ref="A923" r:id="rId922"/>
     <hyperlink ref="A924" r:id="rId923"/>
+    <hyperlink ref="A925" r:id="rId924"/>
+    <hyperlink ref="A926" r:id="rId925"/>
+    <hyperlink ref="A927" r:id="rId926"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -26424,7 +26517,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -26457,62 +26550,122 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>2184</v>
+        <v>2189</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>25</v>
+        <v>185</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>435</v>
+        <v>8</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>25</v>
+        <v>2190</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>25</v>
+        <v>2191</v>
       </c>
       <c r="F2" s="2">
-        <v>46311.226388888885</v>
+        <v>46312.84097222222</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>2185</v>
+        <v>2192</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>290</v>
+        <v>25</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>48</v>
+        <v>435</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>2186</v>
+        <v>25</v>
       </c>
       <c r="F3" s="2">
-        <v>46311.694444444445</v>
+        <v>46314.865277777775</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>2187</v>
+        <v>2193</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>1610</v>
+        <v>25</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>190</v>
+        <v>435</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>44</v>
+        <v>25</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>2188</v>
+        <v>25</v>
       </c>
       <c r="F4" s="2">
-        <v>46311.51041666667</v>
+        <v>46313.80416666667</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>2194</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F5" s="2">
+        <v>46313.4625</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>2195</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>2137</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>695</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>2196</v>
+      </c>
+      <c r="F6" s="2">
+        <v>46314.54791666666</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>2197</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>576</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>659</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>2198</v>
+      </c>
+      <c r="F7" s="2">
+        <v>46313.54236111111</v>
       </c>
     </row>
   </sheetData>
@@ -26520,6 +26673,9 @@
     <hyperlink ref="A2" r:id="rId1"/>
     <hyperlink ref="A3" r:id="rId2"/>
     <hyperlink ref="A4" r:id="rId3"/>
+    <hyperlink ref="A5" r:id="rId4"/>
+    <hyperlink ref="A6" r:id="rId5"/>
+    <hyperlink ref="A7" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-10-20 15:57
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4672" uniqueCount="2199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4692" uniqueCount="2207">
   <si>
     <t>link</t>
   </si>
@@ -6615,6 +6615,30 @@
   </si>
   <si>
     <t>78600020057</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/aluksne-and-reg/zeltinu-pag/bbllii.html</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/gulbene-and-reg/belavas-pag/gcmhx.html</t>
+  </si>
+  <si>
+    <t>50440070260</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/jekabpils-and-reg/elksnu-pag/dfpdg.html</t>
+  </si>
+  <si>
+    <t>56580020134</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/tukums-and-reg/tukums/jigbf.html</t>
+  </si>
+  <si>
+    <t>26 600 €</t>
+  </si>
+  <si>
+    <t>90500080009</t>
   </si>
 </sst>
 </file>
@@ -7027,7 +7051,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F927"/>
+  <dimension ref="A1:F933"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -25576,6 +25600,126 @@
       </c>
       <c r="F927" s="2">
         <v>46311.51041666667</v>
+      </c>
+    </row>
+    <row r="928" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A928" s="3" t="s">
+        <v>2189</v>
+      </c>
+      <c r="B928" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="C928" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D928" s="4" t="s">
+        <v>2190</v>
+      </c>
+      <c r="E928" s="4" t="s">
+        <v>2191</v>
+      </c>
+      <c r="F928" s="2">
+        <v>46312.84097222222</v>
+      </c>
+    </row>
+    <row r="929" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A929" s="3" t="s">
+        <v>2192</v>
+      </c>
+      <c r="B929" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C929" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D929" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E929" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F929" s="2">
+        <v>46314.865277777775</v>
+      </c>
+    </row>
+    <row r="930" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A930" s="3" t="s">
+        <v>2193</v>
+      </c>
+      <c r="B930" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C930" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D930" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E930" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F930" s="2">
+        <v>46313.80416666667</v>
+      </c>
+    </row>
+    <row r="931" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A931" s="3" t="s">
+        <v>2194</v>
+      </c>
+      <c r="B931" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C931" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D931" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E931" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F931" s="2">
+        <v>46313.4625</v>
+      </c>
+    </row>
+    <row r="932" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A932" s="3" t="s">
+        <v>2195</v>
+      </c>
+      <c r="B932" s="4" t="s">
+        <v>2137</v>
+      </c>
+      <c r="C932" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="D932" s="4" t="s">
+        <v>695</v>
+      </c>
+      <c r="E932" s="4" t="s">
+        <v>2196</v>
+      </c>
+      <c r="F932" s="2">
+        <v>46314.54791666666</v>
+      </c>
+    </row>
+    <row r="933" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A933" s="3" t="s">
+        <v>2197</v>
+      </c>
+      <c r="B933" s="4" t="s">
+        <v>576</v>
+      </c>
+      <c r="C933" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="D933" s="4" t="s">
+        <v>659</v>
+      </c>
+      <c r="E933" s="4" t="s">
+        <v>2198</v>
+      </c>
+      <c r="F933" s="2">
+        <v>46313.54236111111</v>
       </c>
     </row>
   </sheetData>
@@ -26506,6 +26650,12 @@
     <hyperlink ref="A925" r:id="rId924"/>
     <hyperlink ref="A926" r:id="rId925"/>
     <hyperlink ref="A927" r:id="rId926"/>
+    <hyperlink ref="A928" r:id="rId927"/>
+    <hyperlink ref="A929" r:id="rId928"/>
+    <hyperlink ref="A930" r:id="rId929"/>
+    <hyperlink ref="A931" r:id="rId930"/>
+    <hyperlink ref="A932" r:id="rId931"/>
+    <hyperlink ref="A933" r:id="rId932"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -26517,7 +26667,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -26550,122 +26700,82 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>2189</v>
+        <v>2199</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>185</v>
+        <v>25</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>8</v>
+        <v>435</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>2190</v>
+        <v>25</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>2191</v>
+        <v>25</v>
       </c>
       <c r="F2" s="2">
-        <v>46312.84097222222</v>
+        <v>46315.19652777778</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>2192</v>
+        <v>2200</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>25</v>
+        <v>185</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>435</v>
+        <v>124</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>25</v>
+        <v>59</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>25</v>
+        <v>2201</v>
       </c>
       <c r="F3" s="2">
-        <v>46314.865277777775</v>
+        <v>46315.674305555556</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>2193</v>
+        <v>2202</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>25</v>
+        <v>1537</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>435</v>
+        <v>127</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>25</v>
+        <v>1135</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>25</v>
+        <v>2203</v>
       </c>
       <c r="F4" s="2">
-        <v>46313.80416666667</v>
+        <v>46315.7375</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>2194</v>
+        <v>2204</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>25</v>
+        <v>2205</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>435</v>
+        <v>376</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>25</v>
+        <v>186</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>25</v>
+        <v>2206</v>
       </c>
       <c r="F5" s="2">
-        <v>46313.4625</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>2195</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>2137</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>256</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>695</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>2196</v>
-      </c>
-      <c r="F6" s="2">
-        <v>46314.54791666666</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
-        <v>2197</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>576</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>294</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>659</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>2198</v>
-      </c>
-      <c r="F7" s="2">
-        <v>46313.54236111111</v>
+        <v>46314.955555555556</v>
       </c>
     </row>
   </sheetData>
@@ -26674,8 +26784,6 @@
     <hyperlink ref="A3" r:id="rId2"/>
     <hyperlink ref="A4" r:id="rId3"/>
     <hyperlink ref="A5" r:id="rId4"/>
-    <hyperlink ref="A6" r:id="rId5"/>
-    <hyperlink ref="A7" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update forest data - 2026-10-21 16:12
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -7051,7 +7051,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F933"/>
+  <dimension ref="A1:F937"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -25720,6 +25720,86 @@
       </c>
       <c r="F933" s="2">
         <v>46313.54236111111</v>
+      </c>
+    </row>
+    <row r="934" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A934" s="3" t="s">
+        <v>2199</v>
+      </c>
+      <c r="B934" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C934" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D934" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E934" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F934" s="2">
+        <v>46315.19652777778</v>
+      </c>
+    </row>
+    <row r="935" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A935" s="3" t="s">
+        <v>2200</v>
+      </c>
+      <c r="B935" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="C935" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="D935" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="E935" s="4" t="s">
+        <v>2201</v>
+      </c>
+      <c r="F935" s="2">
+        <v>46315.674305555556</v>
+      </c>
+    </row>
+    <row r="936" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A936" s="3" t="s">
+        <v>2202</v>
+      </c>
+      <c r="B936" s="4" t="s">
+        <v>1537</v>
+      </c>
+      <c r="C936" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="D936" s="4" t="s">
+        <v>1135</v>
+      </c>
+      <c r="E936" s="4" t="s">
+        <v>2203</v>
+      </c>
+      <c r="F936" s="2">
+        <v>46315.7375</v>
+      </c>
+    </row>
+    <row r="937" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A937" s="3" t="s">
+        <v>2204</v>
+      </c>
+      <c r="B937" s="4" t="s">
+        <v>2205</v>
+      </c>
+      <c r="C937" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="D937" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="E937" s="4" t="s">
+        <v>2206</v>
+      </c>
+      <c r="F937" s="2">
+        <v>46314.955555555556</v>
       </c>
     </row>
   </sheetData>
@@ -26656,6 +26736,10 @@
     <hyperlink ref="A931" r:id="rId930"/>
     <hyperlink ref="A932" r:id="rId931"/>
     <hyperlink ref="A933" r:id="rId932"/>
+    <hyperlink ref="A934" r:id="rId933"/>
+    <hyperlink ref="A935" r:id="rId934"/>
+    <hyperlink ref="A936" r:id="rId935"/>
+    <hyperlink ref="A937" r:id="rId936"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -26667,7 +26751,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -26698,93 +26782,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
-        <v>2199</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>435</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="F2" s="2">
-        <v>46315.19652777778</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>2200</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>185</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>124</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>2201</v>
-      </c>
-      <c r="F3" s="2">
-        <v>46315.674305555556</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>2202</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>1537</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>1135</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>2203</v>
-      </c>
-      <c r="F4" s="2">
-        <v>46315.7375</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>2204</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>2205</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>376</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>2206</v>
-      </c>
-      <c r="F5" s="2">
-        <v>46314.955555555556</v>
-      </c>
-    </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1"/>
-    <hyperlink ref="A3" r:id="rId2"/>
-    <hyperlink ref="A4" r:id="rId3"/>
-    <hyperlink ref="A5" r:id="rId4"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update forest data - 2026-10-22 16:10
</commit_message>
<xml_diff>
--- a/forests-scraped.xlsx
+++ b/forests-scraped.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4692" uniqueCount="2207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4702" uniqueCount="2213">
   <si>
     <t>link</t>
   </si>
@@ -6639,6 +6639,24 @@
   </si>
   <si>
     <t>90500080009</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/valka-and-reg/smiltenes-pag/kjhlg.html</t>
+  </si>
+  <si>
+    <t>950 000 €</t>
+  </si>
+  <si>
+    <t>166 ha.</t>
+  </si>
+  <si>
+    <t>36840030155</t>
+  </si>
+  <si>
+    <t>https://www.ss.com/msg/lv/real-estate/wood/valmiera-and-reg/mazsalaca/nigoo.html</t>
+  </si>
+  <si>
+    <t>96310030005</t>
   </si>
 </sst>
 </file>
@@ -26751,7 +26769,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -26782,7 +26800,51 @@
         <v>5</v>
       </c>
     </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>2207</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>2208</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>2209</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>2210</v>
+      </c>
+      <c r="F2" s="2">
+        <v>46317.53611111111</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>2211</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>396</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>2212</v>
+      </c>
+      <c r="F3" s="2">
+        <v>46317.46041666667</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1"/>
+    <hyperlink ref="A3" r:id="rId2"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>